<commit_message>
Write the shop code from the sources instead of shipping one
The bundled template carried FW430, so a report built from another branch's
exports would have gone out under this branch's code. The code is now read from
the Shop ID the CACO exports state and written into the header, and the shipped
template carries none — which is what makes it usable by any branch rather than
only this one.

A report saved earlier keeps its shop, so re-downloading it from the history
reproduces the same header.

A template uploaded from the interface may still carry a code of its own; that
is left alone when the sources name none, and the existing mismatch check still
compares the two.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N9rz3gZBH9DhH55btFHsLb
</commit_message>
<xml_diff>
--- a/src/assets/daily-template.xlsx
+++ b/src/assets/daily-template.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="20">
   <si>
     <t>تقرير مبيعات المعارض اليومي</t>
   </si>
@@ -26,9 +26,6 @@
   </si>
   <si>
     <t>كود المعرض</t>
-  </si>
-  <si>
-    <t>FW430</t>
   </si>
   <si>
     <t>مشرف المعرض</t>
@@ -1068,41 +1065,39 @@
       <c r="C2" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="10" t="s">
-        <v>3</v>
-      </c>
+      <c r="D2" s="10"/>
       <c r="E2" s="11"/>
     </row>
     <row r="3" ht="49.5" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B3" s="9"/>
       <c r="C3" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D3" s="13"/>
       <c r="E3" s="13"/>
     </row>
     <row r="4" ht="36" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="14" t="s">
         <v>6</v>
-      </c>
-      <c r="B4" s="14" t="s">
-        <v>7</v>
       </c>
       <c r="C4" s="15"/>
       <c r="D4" s="16" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E4" s="17"/>
     </row>
     <row r="5" ht="51.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="18" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="19" t="s">
         <v>9</v>
-      </c>
-      <c r="B5" s="19" t="s">
-        <v>10</v>
       </c>
       <c r="C5" s="20"/>
       <c r="D5" s="21"/>
@@ -1111,7 +1106,7 @@
     <row r="6" ht="51.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="23"/>
       <c r="B6" s="24" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C6" s="25"/>
       <c r="D6" s="26"/>
@@ -1120,7 +1115,7 @@
     <row r="7" ht="51.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="28"/>
       <c r="B7" s="29" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C7" s="30"/>
       <c r="D7" s="31"/>
@@ -1128,22 +1123,22 @@
     </row>
     <row r="8" ht="51.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="18" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C8" s="20"/>
       <c r="D8" s="33"/>
       <c r="E8" s="22"/>
       <c r="H8" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9" ht="51.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="23"/>
       <c r="B9" s="24" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C9" s="25"/>
       <c r="D9" s="26"/>
@@ -1152,30 +1147,30 @@
     <row r="10" ht="51.75" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="28"/>
       <c r="B10" s="29" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C10" s="30"/>
       <c r="D10" s="31"/>
       <c r="E10" s="32"/>
       <c r="J10" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="11" ht="47.25" customHeight="1" spans="1:28" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="34" t="s">
+        <v>15</v>
+      </c>
+      <c r="B11" s="34" t="s">
         <v>16</v>
       </c>
-      <c r="B11" s="34" t="s">
+      <c r="C11" s="34" t="s">
         <v>17</v>
       </c>
-      <c r="C11" s="34" t="s">
+      <c r="D11" s="34" t="s">
         <v>18</v>
       </c>
-      <c r="D11" s="34" t="s">
+      <c r="E11" s="35" t="s">
         <v>19</v>
-      </c>
-      <c r="E11" s="35" t="s">
-        <v>20</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="36"/>

</xml_diff>

<commit_message>
Daily template: write every colour and font itself, so it looks the same without its theme
The template's fills were theme colours (accent + tint) and its headings used
the theme's heading font. A copy opened without its theme part — a mail gateway
that rebuilds attachments, for one — fell back to Excel's default theme: grey
headers, a green payment row, Calibri Light instead of Cambria.

Every theme colour is now the RGB it resolves to in the template's own theme
(Office 2007: green header EBF1DE, blue labels B9CDE5, khaki headings DDD9C3,
peach payment row FCD5B5, blue total C6D9F1), and every font carries its own
name with no theme scheme. Layout, cells, formulas, images unchanged.

Test: templateAsset (2; both fail on the previous template). vitest 328/328.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014KNtaQPK57mZ4cNNFEwgVw
</commit_message>
<xml_diff>
--- a/src/assets/daily-template.xlsx
+++ b/src/assets/daily-template.xlsx
@@ -88,61 +88,53 @@
   </numFmts>
   <fonts count="12" x14ac:knownFonts="1">
     <font>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <family val="2"/>
-      <scheme val="minor"/>
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
     <font>
       <charset val="178"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <family val="2"/>
-      <scheme val="minor"/>
       <sz val="12"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <family val="2"/>
-      <scheme val="minor"/>
       <sz val="18"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <family val="1"/>
-      <scheme val="major"/>
       <sz val="14"/>
       <name val="Cambria"/>
     </font>
     <font>
       <b/>
       <family val="1"/>
-      <scheme val="major"/>
       <sz val="14"/>
       <name val="Cambria"/>
     </font>
     <font>
       <b/>
       <family val="1"/>
-      <scheme val="major"/>
       <sz val="22"/>
       <name val="Cambria"/>
     </font>
     <font>
       <b/>
       <family val="1"/>
-      <scheme val="major"/>
       <sz val="16"/>
       <name val="Cambria"/>
     </font>
     <font>
       <b/>
       <family val="2"/>
-      <scheme val="minor"/>
       <sz val="16"/>
       <name val="Calibri"/>
     </font>
@@ -150,14 +142,12 @@
       <b/>
       <charset val="178"/>
       <family val="2"/>
-      <scheme val="minor"/>
       <sz val="14"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
       <family val="2"/>
-      <scheme val="minor"/>
       <sz val="22"/>
       <name val="Calibri"/>
     </font>
@@ -165,7 +155,6 @@
       <b/>
       <charset val="178"/>
       <family val="2"/>
-      <scheme val="minor"/>
       <sz val="18"/>
       <name val="Calibri"/>
     </font>
@@ -173,7 +162,6 @@
       <b/>
       <charset val="178"/>
       <family val="2"/>
-      <scheme val="minor"/>
       <sz val="26"/>
       <name val="Calibri"/>
     </font>
@@ -187,43 +175,43 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="1"/>
+        <fgColor rgb="FF000000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.7999816888943144"/>
+        <fgColor rgb="FFEBF1DE"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.5999938962981048"/>
+        <fgColor rgb="FFB9CDE5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0"/>
+        <fgColor rgb="FFFFFFFF"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="2" tint="-0.0999786370433668"/>
+        <fgColor rgb="FFDDD9C3"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.5999938962981048"/>
+        <fgColor rgb="FFFCD5B5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="3" tint="0.7999816888943144"/>
+        <fgColor rgb="FFC6D9F1"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>

</xml_diff>